<commit_message>
Saving changes before rebase
</commit_message>
<xml_diff>
--- a/simsek_EX3A_tables.xlsx
+++ b/simsek_EX3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sultansimsek/DATA_Labs/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFFE9B06-CFAB-8E41-B57D-F62A79CEB6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667F93AF-7875-B74D-A081-7E6161ACF103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" activeTab="4" xr2:uid="{0BF8A9BA-4EEE-D74A-B843-16397CF26375}"/>
+    <workbookView xWindow="16040" yWindow="760" windowWidth="14200" windowHeight="17260" activeTab="4" xr2:uid="{0BF8A9BA-4EEE-D74A-B843-16397CF26375}"/>
   </bookViews>
   <sheets>
     <sheet name="Clients" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>Client ID</t>
   </si>
@@ -91,12 +91,39 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Jane Doe</t>
+  </si>
+  <si>
+    <t>111 111 11 11</t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>Nora</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t>1.1.1</t>
+  </si>
+  <si>
+    <t>30 mins</t>
+  </si>
+  <si>
+    <t>Venmo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -145,11 +172,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFDB02CA-B539-EF42-AFCA-D324AB111137}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -504,6 +533,20 @@
         <v>3</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -511,8 +554,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25071E85-9446-E64F-96B6-FD679E181846}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="14.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -531,6 +577,23 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -538,7 +601,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7C75228-2459-1948-A643-AF9374B5AF17}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -561,6 +624,26 @@
         <v>12</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C2" s="4">
+        <v>46023</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="5">
+        <v>15</v>
+      </c>
+      <c r="F2">
+        <v>123456</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -568,7 +651,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC26F39-3CCC-9440-8856-FE40764E38C9}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -589,6 +672,20 @@
         <v>15</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>123456</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46023</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -607,6 +704,14 @@
         <v>12</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2">
+        <v>123456</v>
+      </c>
+    </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
         <v>16</v>

</xml_diff>